<commit_message>
fix: terminate program at lose/win
</commit_message>
<xml_diff>
--- a/Main/Tests/Integrated Tests/integrated_tests.xlsx
+++ b/Main/Tests/Integrated Tests/integrated_tests.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mortrpestl\Desktop\Archives\mortrpestl\The UPper Hand\1st Year\1st Sem\CS11\cs11project\cs11-project-jugemu-jugemu\Tests\Integrated Tests\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mortrpestl\Desktop\Archives\mortrpestl\The UPper Hand\1st Year\1st Sem\CS11\cs11project\cs11-project-jugemu-jugemu\Main\Tests\Integrated Tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BEBDBBC-F76A-4602-B43C-7052C3FDDAD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D51056D-66AF-4407-8E53-2770E87A8B57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>